<commit_message>
Add RDQA Web Tool link to all Tiko application documents
Added the live R/Shiny RDQA Web Tool link
(https://dnfxdz-raymond-wayesu.shinyapps.io/rdqa-web-tool/)
alongside the existing demo dashboard link in all three documents,
with an explanation of the difference between the two:

- Demo dashboard (rdqa-demo.vercel.app): static Next.js website
  showcasing methodology and sample outputs
- RDQA Web Tool (shinyapps.io): live interactive R/Shiny app with
  real-time VF computation, DHIS2 integration, and report generation

Files updated:
- Technical Proposal (.docx): Executive Summary, Section 3.7, footer
- Inception Report (.pptx): Slides 1, 9, 12
- Budget (.xlsx): Both Budget Summary and Monthly Breakdown sheets

Note: The PDF needs to be regenerated locally from the updated DOCX.

https://claude.ai/code/session_015BtjMoQbpeJ26zz4ypTTxf
</commit_message>
<xml_diff>
--- a/docs/Tiko_RDQA_Budget_2026.xlsx
+++ b/docs/Tiko_RDQA_Budget_2026.xlsx
@@ -706,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="29" min="1" max="1"/>
@@ -736,7 +736,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="26.85" customHeight="1" s="30">
       <c r="A5" s="34" t="inlineStr">
         <is>
@@ -1455,7 +1454,6 @@
         <v/>
       </c>
     </row>
-    <row r="38"/>
     <row r="39" ht="15" customHeight="1" s="30">
       <c r="A39" s="42" t="n"/>
       <c r="B39" s="42" t="inlineStr">
@@ -1488,7 +1486,6 @@
         <v/>
       </c>
     </row>
-    <row r="41"/>
     <row r="42" ht="17.35" customHeight="1" s="30">
       <c r="A42" s="45" t="n"/>
       <c r="B42" s="45" t="inlineStr">
@@ -1504,7 +1501,6 @@
         <v/>
       </c>
     </row>
-    <row r="43"/>
     <row r="44" ht="15" customHeight="1" s="30">
       <c r="A44" s="49" t="inlineStr">
         <is>
@@ -1584,6 +1580,18 @@
       <c r="C55" s="52" t="inlineStr">
         <is>
           <t>https://rdqa-demo.vercel.app/</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="51" t="inlineStr">
+        <is>
+          <t>RDQA Web Tool (R/Shiny):</t>
+        </is>
+      </c>
+      <c r="C56" s="52" t="inlineStr">
+        <is>
+          <t>https://dnfxdz-raymond-wayesu.shinyapps.io/rdqa-web-tool/</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="32" customWidth="1" style="29" min="1" max="1"/>
@@ -1632,7 +1640,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="30">
       <c r="A3" s="34" t="inlineStr">
         <is>
@@ -2230,6 +2237,18 @@
       <c r="C18" s="52" t="inlineStr">
         <is>
           <t>https://rdqa-demo.vercel.app/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="51" t="inlineStr">
+        <is>
+          <t>RDQA Web Tool (R/Shiny):</t>
+        </is>
+      </c>
+      <c r="C19" s="52" t="inlineStr">
+        <is>
+          <t>https://dnfxdz-raymond-wayesu.shinyapps.io/rdqa-web-tool/</t>
         </is>
       </c>
     </row>

</xml_diff>